<commit_message>
chg: Prep for D4.1: Ordnance and weather
</commit_message>
<xml_diff>
--- a/MISSION INFORMATION/OPAC Ordnance.xlsx
+++ b/MISSION INFORMATION/OPAC Ordnance.xlsx
@@ -856,7 +856,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1041,7 +1041,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1461,7 +1461,7 @@
       <c r="R1" s="80"/>
       <c r="S1" s="80"/>
       <c r="T1" s="72" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="39.75" customHeight="1">
@@ -1788,7 +1788,9 @@
       <c r="F11" s="56"/>
       <c r="G11" s="56"/>
       <c r="H11" s="56"/>
-      <c r="I11" s="56"/>
+      <c r="I11" s="56">
+        <v>2</v>
+      </c>
       <c r="J11" s="56"/>
       <c r="K11" s="56"/>
       <c r="L11" s="56"/>
@@ -1801,7 +1803,7 @@
       <c r="S11" s="57"/>
       <c r="T11" s="71">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1827,7 +1829,9 @@
       <c r="H12" s="51">
         <v>2</v>
       </c>
-      <c r="I12" s="51"/>
+      <c r="I12" s="51">
+        <v>8</v>
+      </c>
       <c r="J12" s="51"/>
       <c r="K12" s="51"/>
       <c r="L12" s="59"/>
@@ -1840,7 +1844,7 @@
       <c r="S12" s="52"/>
       <c r="T12" s="71">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -2031,7 +2035,9 @@
         <v>4</v>
       </c>
       <c r="H18" s="51"/>
-      <c r="I18" s="51"/>
+      <c r="I18" s="51">
+        <v>2</v>
+      </c>
       <c r="J18" s="51"/>
       <c r="K18" s="51"/>
       <c r="L18" s="51"/>
@@ -2044,7 +2050,7 @@
       <c r="S18" s="52"/>
       <c r="T18" s="53">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="15.75" thickBot="1">

</xml_diff>

<commit_message>
chg: Updated ordnance for D4.2
</commit_message>
<xml_diff>
--- a/MISSION INFORMATION/OPAC Ordnance.xlsx
+++ b/MISSION INFORMATION/OPAC Ordnance.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
-    <sheet name="D9 -&gt;" sheetId="2" r:id="rId1"/>
+    <sheet name="D1 -&gt;" sheetId="2" r:id="rId1"/>
     <sheet name="D1-D8" sheetId="1" r:id="rId2"/>
     <sheet name="Ark3" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -856,7 +856,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1041,7 +1041,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1461,7 +1461,7 @@
       <c r="R1" s="80"/>
       <c r="S1" s="80"/>
       <c r="T1" s="72" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="39.75" customHeight="1">
@@ -1756,7 +1756,9 @@
       <c r="G10" s="51"/>
       <c r="H10" s="51"/>
       <c r="I10" s="51"/>
-      <c r="J10" s="51"/>
+      <c r="J10" s="51">
+        <v>3</v>
+      </c>
       <c r="K10" s="51"/>
       <c r="L10" s="59"/>
       <c r="M10" s="51"/>
@@ -1768,7 +1770,7 @@
       <c r="S10" s="52"/>
       <c r="T10" s="71">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1832,7 +1834,9 @@
       <c r="I12" s="51">
         <v>8</v>
       </c>
-      <c r="J12" s="51"/>
+      <c r="J12" s="51">
+        <v>3</v>
+      </c>
       <c r="K12" s="51"/>
       <c r="L12" s="59"/>
       <c r="M12" s="51"/>
@@ -1844,7 +1848,7 @@
       <c r="S12" s="52"/>
       <c r="T12" s="71">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:20">

</xml_diff>

<commit_message>
chg: Update ordnance, VID intsum and JFC D&G for D5
</commit_message>
<xml_diff>
--- a/MISSION INFORMATION/OPAC Ordnance.xlsx
+++ b/MISSION INFORMATION/OPAC Ordnance.xlsx
@@ -856,7 +856,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1041,7 +1041,7 @@
         <xdr:cNvPr id="2" name="TekstSylinder 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1461,7 +1461,7 @@
       <c r="R1" s="80"/>
       <c r="S1" s="80"/>
       <c r="T1" s="72" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="39.75" customHeight="1">
@@ -1759,7 +1759,9 @@
       <c r="J10" s="51">
         <v>3</v>
       </c>
-      <c r="K10" s="51"/>
+      <c r="K10" s="51">
+        <v>4</v>
+      </c>
       <c r="L10" s="59"/>
       <c r="M10" s="51"/>
       <c r="N10" s="51"/>
@@ -1770,7 +1772,7 @@
       <c r="S10" s="52"/>
       <c r="T10" s="71">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1903,7 +1905,9 @@
       <c r="H14" s="51"/>
       <c r="I14" s="51"/>
       <c r="J14" s="51"/>
-      <c r="K14" s="51"/>
+      <c r="K14" s="51">
+        <v>3</v>
+      </c>
       <c r="L14" s="59"/>
       <c r="M14" s="51"/>
       <c r="N14" s="51"/>
@@ -1914,7 +1918,7 @@
       <c r="S14" s="52"/>
       <c r="T14" s="71">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -2043,7 +2047,9 @@
         <v>2</v>
       </c>
       <c r="J18" s="51"/>
-      <c r="K18" s="51"/>
+      <c r="K18" s="51">
+        <v>4</v>
+      </c>
       <c r="L18" s="51"/>
       <c r="M18" s="51"/>
       <c r="N18" s="51"/>
@@ -2054,7 +2060,7 @@
       <c r="S18" s="52"/>
       <c r="T18" s="53">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="15.75" thickBot="1">

</xml_diff>